<commit_message>
refactor: keep HazardEvent in PublicSchema, remove from AidOps
HazardEvent is a universal concept (disasters, emergencies, economic shocks)
relevant across domains, not specific to humanitarian assessment instruments.
It stays in PS as a subtype of Event alongside PaymentEvent, VitalEvent, etc.

Removed: 1 concept, 5 properties, 3 vocabularies, 2 bibliography entries.
Edited: iasc-mira and iom-dtm bibliography (drop triggering_hazard_event
from informs since it now cross-references PS via vendor).

AidOps now: 3 concepts, 99 properties, 22 vocabularies, 19 bibliography.
</commit_message>
<xml_diff>
--- a/site/public/AnthropometricProfile-definition.xlsx
+++ b/site/public/AnthropometricProfile-definition.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>17 fields defined</t>
+          <t>27 fields defined</t>
         </is>
       </c>
     </row>
@@ -670,17 +670,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="43" customWidth="1" min="11" max="11"/>
@@ -752,70 +752,58 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>height</t>
+          <t>identifiers</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>concept:Identifier</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>The current body height or length of the person, measured in centimeters. For children under 2 years, this is recumbent length; for older children and adults, standing height.</t>
+          <t>Identifiers carried by this entity, such as national ID numbers, program IDs, or identifiers asserted by an identity document.</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>La taille ou longueur corporelle actuelle de la personne, mesurée en centimètres. Pour les enfants de moins de 2 ans, il s'agit de la longueur couchée; pour les enfants plus âgés et les adultes, la taille debout.</t>
+          <t>Identifiants portés par cette entité, tels que numéros d'identité nationale, identifiants de programme ou identifiants attestés par un document d'identité.</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>La talla o longitud corporal actual de la persona, medida en centímetros. Para niños menores de 2 años, es la longitud en decúbito; para niños mayores y adultos, la talla de pie.</t>
+          <t>Identificadores que porta esta entidad, como números de identidad nacional, ID de programa o identificadores acreditados por un documento de identidad.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr"/>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>sensitive</t>
-        </is>
-      </c>
+          <t>normative</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="n"/>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K2" s="8" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4, child_5_17, adult</t>
-        </is>
-      </c>
-      <c r="L2" s="8" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="n"/>
+      <c r="L2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>body_weight</t>
+          <t>subject</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>concept:Party</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
@@ -825,17 +813,17 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>The current body weight of the person, measured in kilograms. Named body_weight to distinguish from birth weight or other weight measures.</t>
+          <t>The person or group that the profile or scoring event is about. Ranged at Party (not Agent) because Profiles observe receivers: persons and organised groups of persons (Household, Family, Farm). Institutional actors (Organizations) are described through their own Organization records, not as subjects of a Profile.</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Le poids corporel actuel de la personne, mesuré en kilogrammes. Nommé body_weight pour le distinguer du poids à la naissance et d'autres mesures de poids.</t>
+          <t>La personne ou le groupe sur lequel porte le profil ou l'événement de notation. Typé sur Party (et non Agent) parce que les Profiles observent des bénéficiaires : personnes et groupes organisés de personnes (Household, Family, Farm). Les acteurs institutionnels (Organizations) sont décrits par leurs propres enregistrements Organization, non comme sujets d'un Profile.</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>El peso corporal actual de la persona, medido en kilogramos. Se denomina body_weight para distinguirlo del peso al nacer y otras medidas de peso.</t>
+          <t>La persona o grupo sobre el que trata el perfil o evento de puntuación. Tipado como Party (no Agent) porque los Profile observan receptores: personas y grupos organizados de personas (Household, Family, Farm). Los actores institucionales (Organizations) se describen mediante sus propios registros Organization, no como sujetos de un Profile.</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr"/>
@@ -844,36 +832,20 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
-        <is>
-          <t>sensitive</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4, child_5_17, adult</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>muac</t>
+          <t>observation_date</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -883,17 +855,17 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>The mid-upper arm circumference (MUAC) of the person, measured in millimeters (unit: mm, typical range 30-300). MUAC is a field screening measure for acute malnutrition in children aged 6-59 months.</t>
+          <t>The date on which the profile data was collected (when the instrument was administered or the measurement taken).</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Le périmètre brachial (PB) de la personne, mesuré en millimètres (unité : mm, plage typique 30-300). Le périmètre brachial est une mesure de dépistage de terrain pour la malnutrition aiguë chez les enfants de 6 à 59 mois.</t>
+          <t>La date à laquelle les données du profil ont été collectées (date d'administration de l'instrument ou de prise de mesure).</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>El perímetro braquial (PB) de la persona, medido en milímetros (unidad: mm, rango típico 30-300). El perímetro braquial es una medida de tamizaje en campo para la desnutrición aguda en niños de 6 a 59 meses.</t>
+          <t>La fecha en que se recopilaron los datos del perfil (fecha en que se administró el instrumento o se tomó la medición).</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
@@ -902,36 +874,20 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>sensitive</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4, adult</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="8" t="n"/>
+      <c r="K4" s="8" t="n"/>
+      <c r="L4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>oedema_present</t>
+          <t>performed_by</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>concept:Agent</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -941,17 +897,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Whether bilateral pitting oedema was observed at the time of measurement. Required for wasting classification under SMART and CMAM protocols: bilateral pitting oedema indicates severe acute malnutrition regardless of MUAC or weight-for-height z-score.</t>
+          <t>The agent (enumerator, field officer, or agency) accountable for administering the instrument or taking the measurement. Typically a Person or an Organization. When a software tool captured or derived the data, record it separately as software_used; performed_by identifies who is responsible, not what ran the capture.</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Indique si un œdème bilatéral prenant le godet a été observé au moment de la mesure. Requis pour la classification de l'émaciation selon les protocoles SMART et PCIMA : un œdème bilatéral prenant le godet indique une malnutrition aiguë sévère indépendamment du périmètre brachial ou du z-score poids-pour-taille.</t>
+          <t>L'agent (enquêteur, agent de terrain ou organisme) responsable de l'administration de l'instrument ou de la prise de mesure. Généralement une Person ou une Organization. Lorsqu'un outil logiciel a capturé ou dérivé les données, enregistrez-le séparément via software_used ; performed_by identifie qui est responsable, et non ce qui a réalisé la capture.</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Indica si se observó edema bilateral con fóvea al momento de la medición. Requerido para la clasificación de emaciación según los protocolos SMART y CMAM: el edema bilateral con fóvea indica desnutrición aguda grave independientemente del perímetro braquial o del puntaje z peso-para-talla.</t>
+          <t>El agente (encuestador, agente de campo u organismo) responsable de administrar el instrumento o tomar la medición. Normalmente una Person o una Organization. Cuando una herramienta de software capturó o derivó los datos, regístrelo por separado mediante software_used; performed_by identifica quién es responsable, no qué ejecutó la captura.</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr"/>
@@ -963,21 +919,17 @@
       <c r="I5" s="10" t="n"/>
       <c r="J5" s="10" t="n"/>
       <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>measurement_type</t>
+          <t>instrument_used</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>concept:Instrument</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -987,24 +939,20 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>How height was measured: recumbent (lying down, for children under two years) or standing. WHO protocols prescribe recumbent length for children under 24 months and standing height from 24 months onward; substituting one for the other introduces a small systematic bias that affects z-score classification.</t>
+          <t>Reference to the instrument (survey form, questionnaire, screening protocol, measurement procedure) administered in this profile record.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Comment la taille a été mesurée : en position couchée (pour les enfants de moins de deux ans) ou debout. Les protocoles de l'OMS prescrivent la longueur couchée pour les enfants de moins de 24 mois et la taille debout à partir de 24 mois ; substituer l'une à l'autre introduit un léger biais systématique qui affecte la classification par z-score.</t>
+          <t>Référence à l'instrument (formulaire d'enquête, questionnaire, protocole de dépistage, procédure de mesure) administré dans cet enregistrement de profil.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Cómo se midió la talla: acostado (para niños menores de dos años) o de pie. Los protocolos de la OMS prescriben longitud en decúbito para niños menores de 24 meses y talla de pie a partir de los 24 meses; sustituir una por otra introduce un pequeño sesgo sistemático que afecta la clasificación por puntaje z.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>measurement-type</t>
-        </is>
-      </c>
+          <t>Referencia al instrumento (formulario de encuesta, cuestionario, protocolo de detección, procedimiento de medición) administrado en este registro de perfil.</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
           <t>draft</t>
@@ -1013,21 +961,17 @@
       <c r="I6" s="8" t="n"/>
       <c r="J6" s="8" t="n"/>
       <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>age_at_measurement_months</t>
+          <t>software_used</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>concept:SoftwareAgent</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -1037,17 +981,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>The subject's age in completed months at the time the measurement was taken. Required for under-five anthropometry because WHO 2006 z-scores are a function of age, sex, and reference population; age now is not interchangeable with age at measurement when the measurement is historical.</t>
+          <t>The software that performed this step, recorded so the result can be reproduced or audited. Distinct from the accountable evaluator or performer (the person or organisation responsible), which is recorded separately.</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>L'âge du sujet en mois révolus au moment de la prise de mesure. Requis pour l'anthropométrie des moins de cinq ans, car les z-scores OMS 2006 sont fonction de l'âge, du sexe et de la population de référence ; l'âge actuel n'est pas interchangeable avec l'âge à la mesure lorsque la mesure est ancienne.</t>
+          <t>Le logiciel qui a effectué cette étape, enregistré afin que le résultat puisse être reproduit ou audité. Distinct de l'évaluateur ou de l'exécutant responsable (la personne ou l'organisme qui en répond), enregistré séparément.</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>La edad del sujeto en meses cumplidos al momento de tomar la medición. Requerido para antropometría en menores de cinco años porque los z-scores OMS 2006 son función de la edad, el sexo y la población de referencia; la edad actual no es intercambiable con la edad al momento de medición cuando la medición es histórica.</t>
+          <t>El software que ejecutó este paso, registrado para que el resultado pueda reproducirse o auditarse. Distinto del evaluador o ejecutor responsable (la persona u organismo que responde), que se registra por separado.</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr"/>
@@ -1059,16 +1003,12 @@
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="10" t="n"/>
       <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>growth_reference</t>
+          <t>administration_mode</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -1083,22 +1023,22 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>The growth reference population used to derive z-scores and band classifications from anthropometric measurements. The WHO Child Growth Standards (2006) are the default for children under five; the WHO Growth Reference (2007) applies to 5-19 year-olds; historical datasets may use the CDC 2000 charts or the NCHS/WHO 1977 reference. Required whenever any derived status (stunting_status, wasting_status, underweight_status, acute_malnutrition_status) is populated.</t>
+          <t>How the instrument was administered to the subject: self-report, proxy-report (someone else answering about the subject), assisted (the subject answering with help), or mixed. Washington Group analytical guidance recommends disaggregating prevalence by administration mode because proxy responses systematically underreport difficulty.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>La population de référence de croissance utilisée pour dériver les z-scores et les classifications par bandes à partir des mesures anthropométriques. Les Normes OMS de croissance de l'enfant (2006) sont la référence par défaut pour les moins de cinq ans ; la Référence OMS de croissance (2007) s'applique aux 5-19 ans ; les jeux de données historiques peuvent utiliser les courbes CDC 2000 ou la référence NCHS/OMS 1977. Requis dès qu'un statut dérivé (stunting_status, wasting_status, underweight_status, acute_malnutrition_status) est renseigné.</t>
+          <t>Comment l'instrument a été administré au sujet : auto-déclaration, déclaration par procuration (quelqu'un d'autre répondant au sujet du sujet), assisté (le sujet répondant avec aide) ou mixte. Les lignes directrices analytiques du Washington Group recommandent de désagréger la prévalence par mode d'administration, car les réponses par procuration sous-déclarent systématiquement la difficulté.</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>La población de referencia de crecimiento utilizada para derivar z-scores y clasificaciones por bandas a partir de mediciones antropométricas. Los Estándares OMS de Crecimiento Infantil (2006) son el valor por defecto para menores de cinco años; la Referencia OMS de Crecimiento (2007) se aplica a los 5-19 años; los conjuntos de datos históricos pueden usar las gráficas CDC 2000 o la referencia NCHS/OMS 1977. Requerido siempre que se complete cualquier estado derivado (stunting_status, wasting_status, underweight_status, acute_malnutrition_status).</t>
+          <t>Cómo se administró el instrumento al sujeto: autoinforme, informe por terceros (otra persona responde sobre el sujeto), asistido (el sujeto responde con ayuda) o mixto. Las directrices analíticas del Washington Group recomiendan desagregar la prevalencia por modo de administración, ya que las respuestas por terceros subestiman sistemáticamente la dificultad.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>growth-reference</t>
+          <t>administration-mode</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1109,21 +1049,17 @@
       <c r="I8" s="8" t="n"/>
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>height_for_age_z</t>
+          <t>respondent</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>concept:Person</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -1133,17 +1069,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>The height-for-age z-score (HAZ) derived from the raw height measurement against the declared growth reference. Values below -2 indicate stunting; below -3 indicate severe stunting under the WHO 2006 standard.</t>
+          <t>The person who provided the answers to the instrument, when different from the subject. Required whenever the administration mode is proxy or assisted.</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Le z-score taille-pour-âge (HAZ) dérivé de la mesure brute de taille par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent un retard de croissance ; inférieures à -3 indiquent un retard sévère selon la norme OMS 2006.</t>
+          <t>La personne qui a fourni les réponses à l'instrument, lorsqu'elle est différente du sujet. Requise lorsque le mode d'administration est par procuration ou assisté.</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>El puntaje z talla-para-edad (HAZ) derivado de la medición bruta de talla respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican retraso del crecimiento; inferiores a -3 indican retraso grave bajo el estándar OMS 2006.</t>
+          <t>La persona que proporcionó las respuestas al instrumento, cuando es distinta del sujeto. Requerida cuando el modo de administración es por terceros o asistido.</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr"/>
@@ -1155,21 +1091,17 @@
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="10" t="n"/>
       <c r="K9" s="10" t="n"/>
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>weight_for_age_z</t>
+          <t>respondent_relationship</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -1179,20 +1111,24 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>The weight-for-age z-score (WAZ) derived from the raw weight measurement against the declared growth reference. Values below -2 indicate underweight; below -3 indicate severe underweight under the WHO 2006 standard.</t>
+          <t>The relationship of the respondent to the subject (parent, spouse, guardian, caregiver, etc.). Uses relationship-type because it describes a person-to-person relationship, not a role within a group. Required whenever the administration mode is proxy or assisted.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Le z-score poids-pour-âge (WAZ) dérivé de la mesure brute de poids par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent une insuffisance pondérale ; inférieures à -3 indiquent une insuffisance sévère selon la norme OMS 2006.</t>
+          <t>La relation du répondant avec le sujet (parent, conjoint, tuteur, aidant, etc.). Utilise relationship-type parce qu'elle décrit une relation entre deux personnes, et non un rôle au sein d'un groupe. Requise lorsque le mode d'administration est par procuration ou assisté.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>El puntaje z peso-para-edad (WAZ) derivado de la medición bruta de peso respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican bajo peso; inferiores a -3 indican bajo peso grave bajo el estándar OMS 2006.</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr"/>
+          <t>La relación del respondiente con el sujeto (padre o madre, cónyuge, tutor, cuidador, etc.). Usa relationship-type porque describe una relación entre personas, no un rol dentro de un grupo. Requerida cuando el modo de administración es por terceros o asistido.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>relationship-type</t>
+        </is>
+      </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
           <t>draft</t>
@@ -1201,41 +1137,37 @@
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
-      <c r="L10" s="8" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>weight_for_height_z</t>
+          <t>items_asked</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>The weight-for-height z-score (WHZ) derived from the raw weight and height measurements against the declared growth reference. Values below -2 indicate wasting; below -3 indicate severe wasting under the WHO 2006 standard.</t>
+          <t>The PublicSchema property IDs that were actually asked during this administration. Lets adopters distinguish items that were asked and declined (answer absent) from items that were not asked at all. When omitted, the item set is assumed to be the default item_set of the instrument used. The intended producer is the form compiler or collection server, which populates this list from the form definition at submission time.</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Le z-score poids-pour-taille (WHZ) dérivé des mesures brutes de poids et de taille par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent une émaciation ; inférieures à -3 indiquent une émaciation sévère selon la norme OMS 2006.</t>
+          <t>Les identifiants de propriétés PublicSchema effectivement posées lors de cette administration. Permet aux adopteurs de distinguer les items posés et refusés (réponse absente) des items qui n'ont pas été posés du tout. En l'absence de cette liste, l'ensemble d'items est présumé correspondre à l'item_set par défaut de l'instrument utilisé. Le producteur prévu est le compilateur de formulaire ou le serveur de collecte, qui remplit cette liste à partir de la définition du formulaire au moment de la soumission.</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>El puntaje z peso-para-talla (WHZ) derivado de las mediciones brutas de peso y talla respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican emaciación; inferiores a -3 indican emaciación grave bajo el estándar OMS 2006.</t>
+          <t>Los identificadores de propiedades PublicSchema realmente preguntados durante esta administración. Permite a los adoptantes distinguir ítems preguntados y rechazados (respuesta ausente) de ítems que no fueron preguntados. Cuando se omite, el conjunto de ítems se asume igual al item_set por defecto del instrumento utilizado. El productor previsto es el compilador de formularios o el servidor de recolección, que completa esta lista a partir de la definición del formulario al momento del envío.</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr"/>
@@ -1247,16 +1179,12 @@
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="10" t="n"/>
       <c r="K11" s="10" t="n"/>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>smart</t>
-        </is>
-      </c>
+      <c r="L11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>bmi_for_age_z</t>
+          <t>height</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1271,17 +1199,17 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>The BMI-for-age z-score (BAZ) derived from height and weight against the declared growth reference. Used under the WHO 2007 reference for school-age children and adolescents (5-19 years) in place of weight-for-height, which does not apply in that age range.</t>
+          <t>The current body height or length of the person, measured in centimeters. For children under 2 years, this is recumbent length; for older children and adults, standing height.</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Le z-score IMC-pour-âge (BAZ) dérivé de la taille et du poids par rapport à la référence de croissance déclarée. Utilisé selon la référence OMS 2007 pour les enfants d'âge scolaire et adolescents (5-19 ans) à la place du poids-pour-taille, qui ne s'applique pas dans cette tranche d'âge.</t>
+          <t>La taille ou longueur corporelle actuelle de la personne, mesurée en centimètres. Pour les enfants de moins de 2 ans, il s'agit de la longueur couchée; pour les enfants plus âgés et les adultes, la taille debout.</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>El puntaje z IMC-para-edad (BAZ) derivado de la talla y el peso respecto a la referencia de crecimiento declarada. Utilizado bajo la referencia OMS 2007 para niños en edad escolar y adolescentes (5-19 años) en lugar del peso-para-talla, que no aplica en ese rango de edad.</t>
+          <t>La talla o longitud corporal actual de la persona, medida en centímetros. Para niños menores de 2 años, es la longitud en decúbito; para niños mayores y adultos, la talla de pie.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr"/>
@@ -1290,9 +1218,21 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>sensitive</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4, child_5_17, adult</t>
+        </is>
+      </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
           <t>smart</t>
@@ -1302,12 +1242,12 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>stunting_status</t>
+          <t>body_weight</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1317,24 +1257,20 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>The stunting classification of the person based on height-for-age z-score (HAZ) relative to the WHO Child Growth Standards.</t>
+          <t>The current body weight of the person, measured in kilograms. Named body_weight to distinguish from birth weight or other weight measures.</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>La classification du retard de croissance de la personne, basée sur le score z taille-pour-âge (HAZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+          <t>Le poids corporel actuel de la personne, mesuré en kilogrammes. Nommé body_weight pour le distinguer du poids à la naissance et d'autres mesures de poids.</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>La clasificación del retraso del crecimiento de la persona, basada en el puntaje z talla-para-la-edad (HAZ) según los estándares de crecimiento infantil de la OMS.</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>malnutrition-severity</t>
-        </is>
-      </c>
+          <t>El peso corporal actual de la persona, medido en kilogramos. Se denomina body_weight para distinguirlo del peso al nacer y otras medidas de peso.</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr"/>
       <c r="H13" s="10" t="inlineStr">
         <is>
           <t>draft</t>
@@ -1352,7 +1288,7 @@
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>infant_0_1, child_2_4</t>
+          <t>infant_0_1, child_2_4, child_5_17, adult</t>
         </is>
       </c>
       <c r="L13" s="10" t="inlineStr">
@@ -1364,12 +1300,12 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>wasting_status</t>
+          <t>muac</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -1379,24 +1315,20 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>The wasting classification of the person based on weight-for-height z-score (WHZ) relative to the WHO Child Growth Standards.</t>
+          <t>The mid-upper arm circumference (MUAC) of the person, measured in millimeters (unit: mm, typical range 30-300). MUAC is a field screening measure for acute malnutrition in children aged 6-59 months.</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>La classification d'émaciation de la personne, basée sur le score z poids-pour-taille (WHZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+          <t>Le périmètre brachial (PB) de la personne, mesuré en millimètres (unité : mm, plage typique 30-300). Le périmètre brachial est une mesure de dépistage de terrain pour la malnutrition aiguë chez les enfants de 6 à 59 mois.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>La clasificación de emaciación de la persona, basada en el puntaje z peso-para-la-talla (WHZ) según los estándares de crecimiento infantil de la OMS.</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>malnutrition-severity</t>
-        </is>
-      </c>
+          <t>El perímetro braquial (PB) de la persona, medido en milímetros (unidad: mm, rango típico 30-300). El perímetro braquial es una medida de tamizaje en campo para la desnutrición aguda en niños de 6 a 59 meses.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr"/>
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>draft</t>
@@ -1414,7 +1346,7 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>infant_0_1, child_2_4</t>
+          <t>infant_0_1, child_2_4, adult</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -1426,12 +1358,12 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>underweight_status</t>
+          <t>oedema_present</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -1441,44 +1373,28 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>The underweight classification of the person based on weight-for-age z-score (WAZ) relative to the WHO Child Growth Standards.</t>
+          <t>Whether bilateral pitting oedema was observed at the time of measurement. Required for wasting classification under SMART and CMAM protocols: bilateral pitting oedema indicates severe acute malnutrition regardless of MUAC or weight-for-height z-score.</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>La classification d'insuffisance pondérale de la personne, basée sur le score z poids-pour-âge (WAZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+          <t>Indique si un œdème bilatéral prenant le godet a été observé au moment de la mesure. Requis pour la classification de l'émaciation selon les protocoles SMART et PCIMA : un œdème bilatéral prenant le godet indique une malnutrition aiguë sévère indépendamment du périmètre brachial ou du z-score poids-pour-taille.</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>La clasificación de insuficiencia ponderal de la persona, basada en el puntaje z peso-para-la-edad (WAZ) según los estándares de crecimiento infantil de la OMS.</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>malnutrition-severity</t>
-        </is>
-      </c>
+          <t>Indica si se observó edema bilateral con fóvea al momento de la medición. Requerido para la clasificación de emaciación según los protocolos SMART y CMAM: el edema bilateral con fóvea indica desnutrición aguda grave independientemente del perímetro braquial o del puntaje z peso-para-talla.</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr"/>
       <c r="H15" s="10" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>sensitive</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4</t>
-        </is>
-      </c>
+      <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
+      <c r="K15" s="10" t="n"/>
       <c r="L15" s="10" t="inlineStr">
         <is>
           <t>smart</t>
@@ -1488,7 +1404,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>acute_malnutrition_status</t>
+          <t>measurement_type</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1503,22 +1419,22 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>The acute malnutrition classification of the person based on mid-upper arm circumference (MUAC) cutoffs defined by the WHO/UNICEF/WFP/UNHCR joint criteria.</t>
+          <t>How height was measured: recumbent (lying down, for children under two years) or standing. WHO protocols prescribe recumbent length for children under 24 months and standing height from 24 months onward; substituting one for the other introduces a small systematic bias that affects z-score classification.</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>La classification de malnutrition aiguë de la personne, basée sur les seuils de périmètre brachial définis par les critères conjoints OMS/UNICEF/PAM/UNHCR.</t>
+          <t>Comment la taille a été mesurée : en position couchée (pour les enfants de moins de deux ans) ou debout. Les protocoles de l'OMS prescrivent la longueur couchée pour les enfants de moins de 24 mois et la taille debout à partir de 24 mois ; substituer l'une à l'autre introduit un léger biais systématique qui affecte la classification par z-score.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>La clasificación de desnutrición aguda de la persona, basada en los puntos de corte de la circunferencia media del brazo definidos por los criterios conjuntos OMS/UNICEF/PMA/ACNUR.</t>
+          <t>Cómo se midió la talla: acostado (para niños menores de dos años) o de pie. Los protocolos de la OMS prescriben longitud en decúbito para niños menores de 24 meses y talla de pie a partir de los 24 meses; sustituir una por otra introduce un pequeño sesgo sistemático que afecta la clasificación por puntaje z.</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>acute-malnutrition-severity</t>
+          <t>measurement-type</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -1526,21 +1442,9 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>sensitive</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4</t>
-        </is>
-      </c>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="inlineStr">
         <is>
           <t>smart</t>
@@ -1550,12 +1454,12 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>muac_band</t>
+          <t>age_at_measurement_months</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -1565,40 +1469,28 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>The red/yellow/green screening band derived from MUAC for children 6-59 months using WHO/UNICEF cutoffs: red (&lt; 115 mm, severe acute malnutrition), yellow (115-124 mm, moderate acute malnutrition), green (&gt;= 125 mm, adequate). This is the field-level colour-coded tape classification used in community screening.</t>
+          <t>The subject's age in completed months at the time the measurement was taken. Required for under-five anthropometry because WHO 2006 z-scores are a function of age, sex, and reference population; age now is not interchangeable with age at measurement when the measurement is historical.</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>La bande de dépistage rouge/jaune/vert dérivée du périmètre brachial pour les enfants de 6 à 59 mois selon les seuils OMS/UNICEF : rouge (&lt; 115 mm, malnutrition aiguë sévère), jaune (115-124 mm, malnutrition aiguë modérée), vert (&gt;= 125 mm, adéquat). Il s'agit de la classification par code couleur du ruban de terrain utilisée dans le dépistage communautaire.</t>
+          <t>L'âge du sujet en mois révolus au moment de la prise de mesure. Requis pour l'anthropométrie des moins de cinq ans, car les z-scores OMS 2006 sont fonction de l'âge, du sexe et de la population de référence ; l'âge actuel n'est pas interchangeable avec l'âge à la mesure lorsque la mesure est ancienne.</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>La banda de tamizaje rojo/amarillo/verde derivada del perímetro braquial para niños de 6 a 59 meses según los puntos de corte OMS/UNICEF: rojo (&lt; 115 mm, desnutrición aguda grave), amarillo (115-124 mm, desnutrición aguda moderada), verde (&gt;= 125 mm, adecuado). Es la clasificación por código de color de la cinta de campo utilizada en el tamizaje comunitario.</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>muac-band</t>
-        </is>
-      </c>
+          <t>La edad del sujeto en meses cumplidos al momento de tomar la medición. Requerido para antropometría en menores de cinco años porque los z-scores OMS 2006 son función de la edad, el sexo y la población de referencia; la edad actual no es intercambiable con la edad al momento de medición cuando la medición es histórica.</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr"/>
       <c r="H17" s="10" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
       <c r="I17" s="10" t="n"/>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>nutrition</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>infant_0_1, child_2_4</t>
-        </is>
-      </c>
+      <c r="J17" s="10" t="n"/>
+      <c r="K17" s="10" t="n"/>
       <c r="L17" s="10" t="inlineStr">
         <is>
           <t>smart</t>
@@ -1608,7 +1500,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>muac_cutoff_rule</t>
+          <t>growth_reference</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -1623,22 +1515,22 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>The population-specific cutoff rule used to classify acute malnutrition from MUAC measurements. MUAC cutoffs differ by population: WHO/UNICEF thresholds for children 6-59 months, z-score based for school-age children and adolescents, Sphere thresholds for pregnant and lactating women. Required whenever acute_malnutrition_status is populated from a MUAC measurement.</t>
+          <t>The growth reference population used to derive z-scores and band classifications from anthropometric measurements. The WHO Child Growth Standards (2006) are the default for children under five; the WHO Growth Reference (2007) applies to 5-19 year-olds; historical datasets may use the CDC 2000 charts or the NCHS/WHO 1977 reference. Required whenever any derived status (stunting_status, wasting_status, underweight_status, acute_malnutrition_status) is populated.</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>La règle de seuil spécifique à la population utilisée pour classer la malnutrition aiguë à partir des mesures de périmètre brachial. Les seuils de périmètre brachial varient selon la population : seuils OMS/UNICEF pour les enfants de 6 à 59 mois, fondés sur le z-score pour les enfants d'âge scolaire et adolescents, seuils Sphere pour les femmes enceintes et allaitantes. Requise dès que acute_malnutrition_status est renseigné à partir d'une mesure de périmètre brachial.</t>
+          <t>La population de référence de croissance utilisée pour dériver les z-scores et les classifications par bandes à partir des mesures anthropométriques. Les Normes OMS de croissance de l'enfant (2006) sont la référence par défaut pour les moins de cinq ans ; la Référence OMS de croissance (2007) s'applique aux 5-19 ans ; les jeux de données historiques peuvent utiliser les courbes CDC 2000 ou la référence NCHS/OMS 1977. Requis dès qu'un statut dérivé (stunting_status, wasting_status, underweight_status, acute_malnutrition_status) est renseigné.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>La regla de corte específica para la población utilizada para clasificar la desnutrición aguda a partir de las mediciones del perímetro braquial. Los cortes de perímetro braquial difieren por población: umbrales OMS/UNICEF para niños de 6 a 59 meses, basados en puntaje z para niños en edad escolar y adolescentes, umbrales Sphere para mujeres embarazadas y lactantes. Requerida siempre que se complete acute_malnutrition_status a partir de una medición del perímetro braquial.</t>
+          <t>La población de referencia de crecimiento utilizada para derivar z-scores y clasificaciones por bandas a partir de mediciones antropométricas. Los Estándares OMS de Crecimiento Infantil (2006) son el valor por defecto para menores de cinco años; la Referencia OMS de Crecimiento (2007) se aplica a los 5-19 años; los conjuntos de datos históricos pueden usar las gráficas CDC 2000 o la referencia NCHS/OMS 1977. Requerido siempre que se complete cualquier estado derivado (stunting_status, wasting_status, underweight_status, acute_malnutrition_status).</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>cutoff-rule</t>
+          <t>growth-reference</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -1650,6 +1542,546 @@
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>height_for_age_z</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>The height-for-age z-score (HAZ) derived from the raw height measurement against the declared growth reference. Values below -2 indicate stunting; below -3 indicate severe stunting under the WHO 2006 standard.</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Le z-score taille-pour-âge (HAZ) dérivé de la mesure brute de taille par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent un retard de croissance ; inférieures à -3 indiquent un retard sévère selon la norme OMS 2006.</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>El puntaje z talla-para-edad (HAZ) derivado de la medición bruta de talla respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican retraso del crecimiento; inferiores a -3 indican retraso grave bajo el estándar OMS 2006.</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>weight_for_age_z</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>The weight-for-age z-score (WAZ) derived from the raw weight measurement against the declared growth reference. Values below -2 indicate underweight; below -3 indicate severe underweight under the WHO 2006 standard.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Le z-score poids-pour-âge (WAZ) dérivé de la mesure brute de poids par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent une insuffisance pondérale ; inférieures à -3 indiquent une insuffisance sévère selon la norme OMS 2006.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>El puntaje z peso-para-edad (WAZ) derivado de la medición bruta de peso respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican bajo peso; inferiores a -3 indican bajo peso grave bajo el estándar OMS 2006.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>weight_for_height_z</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>The weight-for-height z-score (WHZ) derived from the raw weight and height measurements against the declared growth reference. Values below -2 indicate wasting; below -3 indicate severe wasting under the WHO 2006 standard.</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Le z-score poids-pour-taille (WHZ) dérivé des mesures brutes de poids et de taille par rapport à la référence de croissance déclarée. Les valeurs inférieures à -2 indiquent une émaciation ; inférieures à -3 indiquent une émaciation sévère selon la norme OMS 2006.</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>El puntaje z peso-para-talla (WHZ) derivado de las mediciones brutas de peso y talla respecto a la referencia de crecimiento declarada. Valores inferiores a -2 indican emaciación; inferiores a -3 indican emaciación grave bajo el estándar OMS 2006.</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="n"/>
+      <c r="J21" s="10" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>bmi_for_age_z</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>The BMI-for-age z-score (BAZ) derived from height and weight against the declared growth reference. Used under the WHO 2007 reference for school-age children and adolescents (5-19 years) in place of weight-for-height, which does not apply in that age range.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Le z-score IMC-pour-âge (BAZ) dérivé de la taille et du poids par rapport à la référence de croissance déclarée. Utilisé selon la référence OMS 2007 pour les enfants d'âge scolaire et adolescents (5-19 ans) à la place du poids-pour-taille, qui ne s'applique pas dans cette tranche d'âge.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>El puntaje z IMC-para-edad (BAZ) derivado de la talla y el peso respecto a la referencia de crecimiento declarada. Utilizado bajo la referencia OMS 2007 para niños en edad escolar y adolescentes (5-19 años) en lugar del peso-para-talla, que no aplica en ese rango de edad.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="8" t="n"/>
+      <c r="K22" s="8" t="n"/>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>stunting_status</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>The stunting classification of the person based on height-for-age z-score (HAZ) relative to the WHO Child Growth Standards.</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>La classification du retard de croissance de la personne, basée sur le score z taille-pour-âge (HAZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>La clasificación del retraso del crecimiento de la persona, basada en el puntaje z talla-para-la-edad (HAZ) según los estándares de crecimiento infantil de la OMS.</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>malnutrition-severity</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>sensitive</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>wasting_status</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>The wasting classification of the person based on weight-for-height z-score (WHZ) relative to the WHO Child Growth Standards.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>La classification d'émaciation de la personne, basée sur le score z poids-pour-taille (WHZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>La clasificación de emaciación de la persona, basada en el puntaje z peso-para-la-talla (WHZ) según los estándares de crecimiento infantil de la OMS.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>malnutrition-severity</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>sensitive</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>underweight_status</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>The underweight classification of the person based on weight-for-age z-score (WAZ) relative to the WHO Child Growth Standards.</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>La classification d'insuffisance pondérale de la personne, basée sur le score z poids-pour-âge (WAZ) par rapport aux normes de croissance de l'enfant de l'OMS.</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>La clasificación de insuficiencia ponderal de la persona, basada en el puntaje z peso-para-la-edad (WAZ) según los estándares de crecimiento infantil de la OMS.</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>malnutrition-severity</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>sensitive</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4</t>
+        </is>
+      </c>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>acute_malnutrition_status</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>The acute malnutrition classification of the person based on mid-upper arm circumference (MUAC) cutoffs defined by the WHO/UNICEF/WFP/UNHCR joint criteria.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>La classification de malnutrition aiguë de la personne, basée sur les seuils de périmètre brachial définis par les critères conjoints OMS/UNICEF/PAM/UNHCR.</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>La clasificación de desnutrición aguda de la persona, basada en los puntos de corte de la circunferencia media del brazo definidos por los criterios conjuntos OMS/UNICEF/PMA/ACNUR.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>acute-malnutrition-severity</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>sensitive</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>muac_band</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>The red/yellow/green screening band derived from MUAC for children 6-59 months using WHO/UNICEF cutoffs: red (&lt; 115 mm, severe acute malnutrition), yellow (115-124 mm, moderate acute malnutrition), green (&gt;= 125 mm, adequate). This is the field-level colour-coded tape classification used in community screening.</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>La bande de dépistage rouge/jaune/vert dérivée du périmètre brachial pour les enfants de 6 à 59 mois selon les seuils OMS/UNICEF : rouge (&lt; 115 mm, malnutrition aiguë sévère), jaune (115-124 mm, malnutrition aiguë modérée), vert (&gt;= 125 mm, adéquat). Il s'agit de la classification par code couleur du ruban de terrain utilisée dans le dépistage communautaire.</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>La banda de tamizaje rojo/amarillo/verde derivada del perímetro braquial para niños de 6 a 59 meses según los puntos de corte OMS/UNICEF: rojo (&lt; 115 mm, desnutrición aguda grave), amarillo (115-124 mm, desnutrición aguda moderada), verde (&gt;= 125 mm, adecuado). Es la clasificación por código de color de la cinta de campo utilizada en el tamizaje comunitario.</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>muac-band</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>nutrition</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>infant_0_1, child_2_4</t>
+        </is>
+      </c>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>muac_cutoff_rule</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>The population-specific cutoff rule used to classify acute malnutrition from MUAC measurements. MUAC cutoffs differ by population: WHO/UNICEF thresholds for children 6-59 months, z-score based for school-age children and adolescents, Sphere thresholds for pregnant and lactating women. Required whenever acute_malnutrition_status is populated from a MUAC measurement.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>La règle de seuil spécifique à la population utilisée pour classer la malnutrition aiguë à partir des mesures de périmètre brachial. Les seuils de périmètre brachial varient selon la population : seuils OMS/UNICEF pour les enfants de 6 à 59 mois, fondés sur le z-score pour les enfants d'âge scolaire et adolescents, seuils Sphere pour les femmes enceintes et allaitantes. Requise dès que acute_malnutrition_status est renseigné à partir d'une mesure de périmètre brachial.</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>La regla de corte específica para la población utilizada para clasificar la desnutrición aguda a partir de las mediciones del perímetro braquial. Los cortes de perímetro braquial difieren por población: umbrales OMS/UNICEF para niños de 6 a 59 meses, basados en puntaje z para niños en edad escolar y adolescentes, umbrales Sphere para mujeres embarazadas y lactantes. Requerida siempre que se complete acute_malnutrition_status a partir de una medición del perímetro braquial.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>cutoff-rule</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
+      <c r="K28" s="8" t="n"/>
+      <c r="L28" s="8" t="inlineStr">
         <is>
           <t>smart</t>
         </is>

</xml_diff>